<commit_message>
Updated message and description and negative test data.
</commit_message>
<xml_diff>
--- a/rules/CORE-000502/negative/01/data/unit-test-coreid-CG0369-negative.xlsx
+++ b/rules/CORE-000502/negative/01/data/unit-test-coreid-CG0369-negative.xlsx
@@ -9,6 +9,7 @@
     <sheet name="supplb.xpt" sheetId="4" r:id="rId4"/>
     <sheet name="relrec.xpt" sheetId="5" r:id="rId5"/>
     <sheet name="co.xpt" sheetId="6" r:id="rId6"/>
+    <sheet name="lb.xpt" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -79,7 +80,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFCC"/>
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -475,7 +476,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -509,16 +510,24 @@
         <v>Comments</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="2" t="str">
+        <v>lb.xpt</v>
+      </c>
+      <c r="B5" s="2" t="str">
+        <v>Laboratory Results</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F2"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -542,10 +551,10 @@
     </row>
     <row r="2">
       <c r="A2" s="2">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="2" t="str">
-        <v>supplb.xpt</v>
+        <v>co.xpt</v>
       </c>
       <c r="C2" s="2" t="str">
         <v>Record</v>
@@ -557,52 +566,12 @@
         <v>RDOMAIN</v>
       </c>
       <c r="F2" s="2" t="str">
-        <v>LB</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="str">
-        <v>relrec.xpt</v>
-      </c>
-      <c r="C3" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D3" s="2">
-        <v>5</v>
-      </c>
-      <c r="E3" s="2" t="str">
-        <v>RDOMAIN</v>
-      </c>
-      <c r="F3" s="2" t="str">
-        <v>LB</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="str">
-        <v>co.xpt</v>
-      </c>
-      <c r="C4" s="2" t="str">
-        <v>Record</v>
-      </c>
-      <c r="D4" s="2">
-        <v>5</v>
-      </c>
-      <c r="E4" s="2" t="str">
-        <v>RDOMAIN</v>
-      </c>
-      <c r="F4" s="2" t="str">
         <v>IS</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1103,4 +1072,955 @@
     <ignoredError numberStoredAsText="1" sqref="A1:M5"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:BJ5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="str">
+        <v>STUDYID</v>
+      </c>
+      <c r="B1" s="3" t="str">
+        <v>DOMAIN</v>
+      </c>
+      <c r="C1" s="3" t="str">
+        <v>USUBJID</v>
+      </c>
+      <c r="D1" s="3" t="str">
+        <v>LBSEQ</v>
+      </c>
+      <c r="E1" s="3" t="str">
+        <v>LBGRPID</v>
+      </c>
+      <c r="F1" s="3" t="str">
+        <v>LBREFID</v>
+      </c>
+      <c r="G1" s="3" t="str">
+        <v>LBSPID</v>
+      </c>
+      <c r="H1" s="3" t="str">
+        <v>LBTESTCD</v>
+      </c>
+      <c r="I1" s="3" t="str">
+        <v>LBTEST</v>
+      </c>
+      <c r="J1" s="3" t="str">
+        <v>LBTSTCND</v>
+      </c>
+      <c r="K1" s="3" t="str">
+        <v>LBBDAGNT</v>
+      </c>
+      <c r="L1" s="3" t="str">
+        <v>LBTSTOPO</v>
+      </c>
+      <c r="M1" s="3" t="str">
+        <v>LBCAT</v>
+      </c>
+      <c r="N1" s="3" t="str">
+        <v>LBSCAT</v>
+      </c>
+      <c r="O1" s="3" t="str">
+        <v>LBORRES</v>
+      </c>
+      <c r="P1" s="3" t="str">
+        <v>LBORRESU</v>
+      </c>
+      <c r="Q1" s="3" t="str">
+        <v>LBRESSCL</v>
+      </c>
+      <c r="R1" s="3" t="str">
+        <v>LBRESTYP</v>
+      </c>
+      <c r="S1" s="3" t="str">
+        <v>LBCOLSRT</v>
+      </c>
+      <c r="T1" s="3" t="str">
+        <v>LBORNRLO</v>
+      </c>
+      <c r="U1" s="3" t="str">
+        <v>LBORNRHI</v>
+      </c>
+      <c r="V1" s="3" t="str">
+        <v>LBLLOD</v>
+      </c>
+      <c r="W1" s="3" t="str">
+        <v>LBSTRESC</v>
+      </c>
+      <c r="X1" s="3" t="str">
+        <v>LBSTRESN</v>
+      </c>
+      <c r="Y1" s="3" t="str">
+        <v>LBSTRESU</v>
+      </c>
+      <c r="Z1" s="3" t="str">
+        <v>LBSTNRLO</v>
+      </c>
+      <c r="AA1" s="3" t="str">
+        <v>LBSTNRHI</v>
+      </c>
+      <c r="AB1" s="3" t="str">
+        <v>LBSTNRC</v>
+      </c>
+      <c r="AC1" s="3" t="str">
+        <v>LBNRIND</v>
+      </c>
+      <c r="AD1" s="3" t="str">
+        <v>LBSTAT</v>
+      </c>
+      <c r="AE1" s="3" t="str">
+        <v>LBREASND</v>
+      </c>
+      <c r="AF1" s="3" t="str">
+        <v>LBNAM</v>
+      </c>
+      <c r="AG1" s="3" t="str">
+        <v>LBLOINC</v>
+      </c>
+      <c r="AH1" s="3" t="str">
+        <v>LBSPEC</v>
+      </c>
+      <c r="AI1" s="3" t="str">
+        <v>LBSPCCND</v>
+      </c>
+      <c r="AJ1" s="3" t="str">
+        <v>LBSPCUFL</v>
+      </c>
+      <c r="AK1" s="3" t="str">
+        <v>LBMETHOD</v>
+      </c>
+      <c r="AL1" s="3" t="str">
+        <v>LBANMETH</v>
+      </c>
+      <c r="AM1" s="3" t="str">
+        <v>LBTMTHSN</v>
+      </c>
+      <c r="AN1" s="3" t="str">
+        <v>LBLOBXFL</v>
+      </c>
+      <c r="AO1" s="3" t="str">
+        <v>LBBLFL</v>
+      </c>
+      <c r="AP1" s="3" t="str">
+        <v>LBFAST</v>
+      </c>
+      <c r="AQ1" s="3" t="str">
+        <v>LBDRVFL</v>
+      </c>
+      <c r="AR1" s="3" t="str">
+        <v>LBTOX</v>
+      </c>
+      <c r="AS1" s="3" t="str">
+        <v>LBTOXGR</v>
+      </c>
+      <c r="AT1" s="3" t="str">
+        <v>LBCLSIG</v>
+      </c>
+      <c r="AU1" s="3" t="str">
+        <v>VISITNUM</v>
+      </c>
+      <c r="AV1" s="3" t="str">
+        <v>VISIT</v>
+      </c>
+      <c r="AW1" s="3" t="str">
+        <v>VISITDY</v>
+      </c>
+      <c r="AX1" s="3" t="str">
+        <v>TAETORD</v>
+      </c>
+      <c r="AY1" s="3" t="str">
+        <v>EPOCH</v>
+      </c>
+      <c r="AZ1" s="3" t="str">
+        <v>LBDTC</v>
+      </c>
+      <c r="BA1" s="3" t="str">
+        <v>LBENDTC</v>
+      </c>
+      <c r="BB1" s="3" t="str">
+        <v>LBDY</v>
+      </c>
+      <c r="BC1" s="3" t="str">
+        <v>LBENDY</v>
+      </c>
+      <c r="BD1" s="3" t="str">
+        <v>LBTPT</v>
+      </c>
+      <c r="BE1" s="3" t="str">
+        <v>LBTPTNUM</v>
+      </c>
+      <c r="BF1" s="3" t="str">
+        <v>LBELTM</v>
+      </c>
+      <c r="BG1" s="3" t="str">
+        <v>LBTPTREF</v>
+      </c>
+      <c r="BH1" s="3" t="str">
+        <v>LBRFTDTC</v>
+      </c>
+      <c r="BI1" s="3" t="str">
+        <v>LBPTFL</v>
+      </c>
+      <c r="BJ1" s="3" t="str">
+        <v>LBPDUR</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="str">
+        <v>Study Identifier</v>
+      </c>
+      <c r="B2" s="5" t="str">
+        <v>Domain Abbreviation</v>
+      </c>
+      <c r="C2" s="5" t="str">
+        <v>Unique Subject Identifier</v>
+      </c>
+      <c r="D2" s="5" t="str">
+        <v>Sequence Number</v>
+      </c>
+      <c r="E2" s="5" t="str">
+        <v>Group ID</v>
+      </c>
+      <c r="F2" s="5" t="str">
+        <v>Specimen ID</v>
+      </c>
+      <c r="G2" s="5" t="str">
+        <v>Sponsor-Defined Identifier</v>
+      </c>
+      <c r="H2" s="5" t="str">
+        <v>Lab Test or Examination Short Name</v>
+      </c>
+      <c r="I2" s="5" t="str">
+        <v>Lab Test or Examination Name</v>
+      </c>
+      <c r="J2" s="5" t="str">
+        <v>Test Condition</v>
+      </c>
+      <c r="K2" s="5" t="str">
+        <v>Binding Agent</v>
+      </c>
+      <c r="L2" s="5" t="str">
+        <v>Test Operational Objective</v>
+      </c>
+      <c r="M2" s="5" t="str">
+        <v>Category for Lab Test</v>
+      </c>
+      <c r="N2" s="5" t="str">
+        <v>Subcategory for Lab Test</v>
+      </c>
+      <c r="O2" s="5" t="str">
+        <v>Result or Finding in Original Units</v>
+      </c>
+      <c r="P2" s="5" t="str">
+        <v>Original Units</v>
+      </c>
+      <c r="Q2" s="5" t="str">
+        <v>Result Scale</v>
+      </c>
+      <c r="R2" s="5" t="str">
+        <v>Result Type</v>
+      </c>
+      <c r="S2" s="5" t="str">
+        <v>Collected Summary Result Type</v>
+      </c>
+      <c r="T2" s="5" t="str">
+        <v>Reference Range Lower Limit in Orig Unit</v>
+      </c>
+      <c r="U2" s="5" t="str">
+        <v>Reference Range Upper Limit in Orig Unit</v>
+      </c>
+      <c r="V2" s="5" t="str">
+        <v>Lower Limit of Detection</v>
+      </c>
+      <c r="W2" s="5" t="str">
+        <v>Character Result/Finding in Std Format</v>
+      </c>
+      <c r="X2" s="5" t="str">
+        <v>Numeric Result/Finding in Standard Units</v>
+      </c>
+      <c r="Y2" s="5" t="str">
+        <v>Standard Units</v>
+      </c>
+      <c r="Z2" s="5" t="str">
+        <v>Reference Range Lower Limit-Std Units</v>
+      </c>
+      <c r="AA2" s="5" t="str">
+        <v>Reference Range Upper Limit-Std Units</v>
+      </c>
+      <c r="AB2" s="5" t="str">
+        <v>Reference Range for Char Rslt-Std Units</v>
+      </c>
+      <c r="AC2" s="5" t="str">
+        <v>Reference Range Indicator</v>
+      </c>
+      <c r="AD2" s="5" t="str">
+        <v>Completion Status</v>
+      </c>
+      <c r="AE2" s="5" t="str">
+        <v>Reason Test Not Done</v>
+      </c>
+      <c r="AF2" s="5" t="str">
+        <v>Vendor Name</v>
+      </c>
+      <c r="AG2" s="5" t="str">
+        <v>LOINC Code</v>
+      </c>
+      <c r="AH2" s="5" t="str">
+        <v>Specimen Type</v>
+      </c>
+      <c r="AI2" s="5" t="str">
+        <v>Specimen Condition</v>
+      </c>
+      <c r="AJ2" s="5" t="str">
+        <v>Specimen Usability for the Test</v>
+      </c>
+      <c r="AK2" s="5" t="str">
+        <v>Method of Test or Examination</v>
+      </c>
+      <c r="AL2" s="5" t="str">
+        <v>Analysis Method</v>
+      </c>
+      <c r="AM2" s="5" t="str">
+        <v>Test Method Sensitivity</v>
+      </c>
+      <c r="AN2" s="5" t="str">
+        <v>Last Observation Before Exposure Flag</v>
+      </c>
+      <c r="AO2" s="5" t="str">
+        <v>Baseline Flag</v>
+      </c>
+      <c r="AP2" s="5" t="str">
+        <v>Fasting Status</v>
+      </c>
+      <c r="AQ2" s="5" t="str">
+        <v>Derived Flag</v>
+      </c>
+      <c r="AR2" s="5" t="str">
+        <v>Toxicity</v>
+      </c>
+      <c r="AS2" s="5" t="str">
+        <v>Standard Toxicity Grade</v>
+      </c>
+      <c r="AT2" s="5" t="str">
+        <v>Clinically Significant, Collected</v>
+      </c>
+      <c r="AU2" s="5" t="str">
+        <v>Visit Number</v>
+      </c>
+      <c r="AV2" s="5" t="str">
+        <v>Visit Name</v>
+      </c>
+      <c r="AW2" s="5" t="str">
+        <v>Planned Study Day of Visit</v>
+      </c>
+      <c r="AX2" s="5" t="str">
+        <v>Planned Order of Element within Arm</v>
+      </c>
+      <c r="AY2" s="5" t="str">
+        <v>Epoch</v>
+      </c>
+      <c r="AZ2" s="5" t="str">
+        <v>Date/Time of Specimen Collection</v>
+      </c>
+      <c r="BA2" s="5" t="str">
+        <v>End Date/Time of Specimen Collection</v>
+      </c>
+      <c r="BB2" s="5" t="str">
+        <v>Study Day of Specimen Collection</v>
+      </c>
+      <c r="BC2" s="5" t="str">
+        <v>Study Day of End of Observation</v>
+      </c>
+      <c r="BD2" s="5" t="str">
+        <v>Planned Time Point Name</v>
+      </c>
+      <c r="BE2" s="5" t="str">
+        <v>Planned Time Point Number</v>
+      </c>
+      <c r="BF2" s="5" t="str">
+        <v>Planned Elapsed Time from Time Point Ref</v>
+      </c>
+      <c r="BG2" s="5" t="str">
+        <v>Time Point Reference</v>
+      </c>
+      <c r="BH2" s="5" t="str">
+        <v>Date/Time of Reference Time Point</v>
+      </c>
+      <c r="BI2" s="5" t="str">
+        <v>Point in Time Flag</v>
+      </c>
+      <c r="BJ2" s="5" t="str">
+        <v>Planned Duration</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="E3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="P3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="Y3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="AA3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="AB3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AC3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AD3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AE3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AF3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AG3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AH3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AI3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AJ3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AK3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AL3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AM3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AN3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AO3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AP3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AQ3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AR3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AS3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AT3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AU3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="AV3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AW3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="AX3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="AY3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AZ3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BA3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BB3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="BC3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="BD3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BE3" s="5" t="str">
+        <v>Num</v>
+      </c>
+      <c r="BF3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BG3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BH3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BI3" s="5" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BJ3" s="5" t="str">
+        <v>Char</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="B4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="C4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="D4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="E4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="F4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="G4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="H4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="I4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="J4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="L4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="M4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="N4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="O4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="P4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="R4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="S4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="T4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="U4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="V4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="W4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="X4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="Y4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="Z4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="AA4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="AB4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AD4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AE4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AF4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AG4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AH4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AI4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AJ4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AK4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AL4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AM4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AN4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AO4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AP4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AQ4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AR4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AS4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AT4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AU4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="AV4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AW4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="AX4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="AY4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="AZ4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BA4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BB4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="BC4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="BD4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BE4" s="5" t="str">
+        <v>8</v>
+      </c>
+      <c r="BF4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BG4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BH4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BI4" s="5" t="str">
+        <v>50</v>
+      </c>
+      <c r="BJ4" s="5" t="str">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="str">
+        <v>CDISC-PILOT-01</v>
+      </c>
+      <c r="B5" s="4" t="str">
+        <v>LB</v>
+      </c>
+      <c r="C5" s="4" t="str">
+        <v>S001</v>
+      </c>
+      <c r="D5" s="4" t="str">
+        <v>320</v>
+      </c>
+      <c r="E5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="F5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="G5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="H5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="I5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="J5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="K5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="L5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="M5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="N5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="O5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="P5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Q5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="R5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="S5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="T5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="U5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="V5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="W5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="X5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Y5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="Z5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AA5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AB5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AC5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AD5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AE5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AF5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AG5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AH5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AI5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AJ5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AK5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AL5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AM5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AN5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AO5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AP5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AQ5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AR5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AS5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AT5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AU5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AV5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AW5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AX5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AY5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="AZ5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BA5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BB5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BC5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BD5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BE5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BF5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BG5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BH5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BI5" s="4" t="str">
+        <v/>
+      </c>
+      <c r="BJ5" s="4" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:BJ5"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed negative test validation.
</commit_message>
<xml_diff>
--- a/rules/CORE-000502/negative/01/data/unit-test-coreid-CG0369-negative.xlsx
+++ b/rules/CORE-000502/negative/01/data/unit-test-coreid-CG0369-negative.xlsx
@@ -39,7 +39,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -65,9 +65,14 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+      <i/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none">
         <bgColor/>
@@ -75,6 +80,12 @@
     </fill>
     <fill>
       <patternFill patternType="gray125">
+        <bgColor/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor/>
       </patternFill>
     </fill>
@@ -110,7 +121,7 @@
   <cellStyleXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="1" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -118,6 +129,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,95 +628,95 @@
       <c r="A2" s="5" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Related Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Identifying Variable</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Identifying Variable Value</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Qualifier Variable Name</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Qualifier Variable Label</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Data Value</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Origin</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Evaluator</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
         <v>50</v>
       </c>
     </row>
@@ -712,7 +724,7 @@
       <c r="A5" s="4" t="str">
         <v>CDISC-PILOT-01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>LB</v>
       </c>
       <c r="C5" s="4" t="str">
@@ -772,71 +784,71 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Related Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Identifying Variable</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Identifying Variable Value</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Relationship Type</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Relationship Identifier</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
         <v>50</v>
       </c>
     </row>
@@ -844,7 +856,7 @@
       <c r="A5" s="4" t="str">
         <v>CDISC-PILOT-01</v>
       </c>
-      <c r="B5" s="6" t="str">
+      <c r="B5" s="4" t="str">
         <v>LB</v>
       </c>
       <c r="C5" s="4" t="str">
@@ -916,125 +928,125 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Related Domain Abbreviation</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Identifying Variable</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Identifying Variable Value</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Comment Reference</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Comment</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Evaluator</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Evaluator Identifier</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Date/Time of Comment</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Study Day of Comment</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="E3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="E3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
         <v>Num</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5">
-        <v>50</v>
-      </c>
-      <c r="E4" s="5">
+      <c r="A4" s="6">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6">
+        <v>50</v>
+      </c>
+      <c r="E4" s="6">
         <v>8</v>
       </c>
-      <c r="F4" s="5">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5">
+      <c r="F4" s="6">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6">
+        <v>50</v>
+      </c>
+      <c r="K4" s="6">
+        <v>50</v>
+      </c>
+      <c r="L4" s="6">
+        <v>50</v>
+      </c>
+      <c r="M4" s="6">
         <v>8</v>
       </c>
     </row>
@@ -1045,7 +1057,7 @@
       <c r="B5" s="4" t="str">
         <v>CO</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="7" t="str">
         <v>IS</v>
       </c>
       <c r="D5" s="4" t="str">
@@ -1267,566 +1279,566 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Group ID</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Specimen ID</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Sponsor-Defined Identifier</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Lab Test or Examination Short Name</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Lab Test or Examination Name</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>Test Condition</v>
       </c>
-      <c r="K2" s="5" t="str">
+      <c r="K2" s="6" t="str">
         <v>Binding Agent</v>
       </c>
-      <c r="L2" s="5" t="str">
+      <c r="L2" s="6" t="str">
         <v>Test Operational Objective</v>
       </c>
-      <c r="M2" s="5" t="str">
+      <c r="M2" s="6" t="str">
         <v>Category for Lab Test</v>
       </c>
-      <c r="N2" s="5" t="str">
+      <c r="N2" s="6" t="str">
         <v>Subcategory for Lab Test</v>
       </c>
-      <c r="O2" s="5" t="str">
+      <c r="O2" s="6" t="str">
         <v>Result or Finding in Original Units</v>
       </c>
-      <c r="P2" s="5" t="str">
+      <c r="P2" s="6" t="str">
         <v>Original Units</v>
       </c>
-      <c r="Q2" s="5" t="str">
+      <c r="Q2" s="6" t="str">
         <v>Result Scale</v>
       </c>
-      <c r="R2" s="5" t="str">
+      <c r="R2" s="6" t="str">
         <v>Result Type</v>
       </c>
-      <c r="S2" s="5" t="str">
+      <c r="S2" s="6" t="str">
         <v>Collected Summary Result Type</v>
       </c>
-      <c r="T2" s="5" t="str">
+      <c r="T2" s="6" t="str">
         <v>Reference Range Lower Limit in Orig Unit</v>
       </c>
-      <c r="U2" s="5" t="str">
+      <c r="U2" s="6" t="str">
         <v>Reference Range Upper Limit in Orig Unit</v>
       </c>
-      <c r="V2" s="5" t="str">
+      <c r="V2" s="6" t="str">
         <v>Lower Limit of Detection</v>
       </c>
-      <c r="W2" s="5" t="str">
+      <c r="W2" s="6" t="str">
         <v>Character Result/Finding in Std Format</v>
       </c>
-      <c r="X2" s="5" t="str">
+      <c r="X2" s="6" t="str">
         <v>Numeric Result/Finding in Standard Units</v>
       </c>
-      <c r="Y2" s="5" t="str">
+      <c r="Y2" s="6" t="str">
         <v>Standard Units</v>
       </c>
-      <c r="Z2" s="5" t="str">
+      <c r="Z2" s="6" t="str">
         <v>Reference Range Lower Limit-Std Units</v>
       </c>
-      <c r="AA2" s="5" t="str">
+      <c r="AA2" s="6" t="str">
         <v>Reference Range Upper Limit-Std Units</v>
       </c>
-      <c r="AB2" s="5" t="str">
+      <c r="AB2" s="6" t="str">
         <v>Reference Range for Char Rslt-Std Units</v>
       </c>
-      <c r="AC2" s="5" t="str">
+      <c r="AC2" s="6" t="str">
         <v>Reference Range Indicator</v>
       </c>
-      <c r="AD2" s="5" t="str">
+      <c r="AD2" s="6" t="str">
         <v>Completion Status</v>
       </c>
-      <c r="AE2" s="5" t="str">
+      <c r="AE2" s="6" t="str">
         <v>Reason Test Not Done</v>
       </c>
-      <c r="AF2" s="5" t="str">
+      <c r="AF2" s="6" t="str">
         <v>Vendor Name</v>
       </c>
-      <c r="AG2" s="5" t="str">
+      <c r="AG2" s="6" t="str">
         <v>LOINC Code</v>
       </c>
-      <c r="AH2" s="5" t="str">
+      <c r="AH2" s="6" t="str">
         <v>Specimen Type</v>
       </c>
-      <c r="AI2" s="5" t="str">
+      <c r="AI2" s="6" t="str">
         <v>Specimen Condition</v>
       </c>
-      <c r="AJ2" s="5" t="str">
+      <c r="AJ2" s="6" t="str">
         <v>Specimen Usability for the Test</v>
       </c>
-      <c r="AK2" s="5" t="str">
+      <c r="AK2" s="6" t="str">
         <v>Method of Test or Examination</v>
       </c>
-      <c r="AL2" s="5" t="str">
+      <c r="AL2" s="6" t="str">
         <v>Analysis Method</v>
       </c>
-      <c r="AM2" s="5" t="str">
+      <c r="AM2" s="6" t="str">
         <v>Test Method Sensitivity</v>
       </c>
-      <c r="AN2" s="5" t="str">
+      <c r="AN2" s="6" t="str">
         <v>Last Observation Before Exposure Flag</v>
       </c>
-      <c r="AO2" s="5" t="str">
+      <c r="AO2" s="6" t="str">
         <v>Baseline Flag</v>
       </c>
-      <c r="AP2" s="5" t="str">
+      <c r="AP2" s="6" t="str">
         <v>Fasting Status</v>
       </c>
-      <c r="AQ2" s="5" t="str">
+      <c r="AQ2" s="6" t="str">
         <v>Derived Flag</v>
       </c>
-      <c r="AR2" s="5" t="str">
+      <c r="AR2" s="6" t="str">
         <v>Toxicity</v>
       </c>
-      <c r="AS2" s="5" t="str">
+      <c r="AS2" s="6" t="str">
         <v>Standard Toxicity Grade</v>
       </c>
-      <c r="AT2" s="5" t="str">
+      <c r="AT2" s="6" t="str">
         <v>Clinically Significant, Collected</v>
       </c>
-      <c r="AU2" s="5" t="str">
+      <c r="AU2" s="6" t="str">
         <v>Visit Number</v>
       </c>
-      <c r="AV2" s="5" t="str">
+      <c r="AV2" s="6" t="str">
         <v>Visit Name</v>
       </c>
-      <c r="AW2" s="5" t="str">
+      <c r="AW2" s="6" t="str">
         <v>Planned Study Day of Visit</v>
       </c>
-      <c r="AX2" s="5" t="str">
+      <c r="AX2" s="6" t="str">
         <v>Planned Order of Element within Arm</v>
       </c>
-      <c r="AY2" s="5" t="str">
+      <c r="AY2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="AZ2" s="5" t="str">
+      <c r="AZ2" s="6" t="str">
         <v>Date/Time of Specimen Collection</v>
       </c>
-      <c r="BA2" s="5" t="str">
+      <c r="BA2" s="6" t="str">
         <v>End Date/Time of Specimen Collection</v>
       </c>
-      <c r="BB2" s="5" t="str">
+      <c r="BB2" s="6" t="str">
         <v>Study Day of Specimen Collection</v>
       </c>
-      <c r="BC2" s="5" t="str">
+      <c r="BC2" s="6" t="str">
         <v>Study Day of End of Observation</v>
       </c>
-      <c r="BD2" s="5" t="str">
+      <c r="BD2" s="6" t="str">
         <v>Planned Time Point Name</v>
       </c>
-      <c r="BE2" s="5" t="str">
+      <c r="BE2" s="6" t="str">
         <v>Planned Time Point Number</v>
       </c>
-      <c r="BF2" s="5" t="str">
+      <c r="BF2" s="6" t="str">
         <v>Planned Elapsed Time from Time Point Ref</v>
       </c>
-      <c r="BG2" s="5" t="str">
+      <c r="BG2" s="6" t="str">
         <v>Time Point Reference</v>
       </c>
-      <c r="BH2" s="5" t="str">
+      <c r="BH2" s="6" t="str">
         <v>Date/Time of Reference Time Point</v>
       </c>
-      <c r="BI2" s="5" t="str">
+      <c r="BI2" s="6" t="str">
         <v>Point in Time Flag</v>
       </c>
-      <c r="BJ2" s="5" t="str">
+      <c r="BJ2" s="6" t="str">
         <v>Planned Duration</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="K3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="L3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="M3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="N3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="O3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="P3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Q3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="R3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="S3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="T3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="U3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="V3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="W3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="X3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="K3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="L3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="M3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="N3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="O3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="P3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Q3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="R3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="S3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="T3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="U3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="V3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="W3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="X3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="Y3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="Z3" s="5" t="str">
+      <c r="Y3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="Z3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AA3" s="5" t="str">
+      <c r="AA3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AB3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AC3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AD3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AE3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AF3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AG3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AH3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AI3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AJ3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AK3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AL3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AM3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AN3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AO3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AP3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AQ3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AR3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AS3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AT3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AU3" s="5" t="str">
+      <c r="AB3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AC3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AD3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AE3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AF3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AG3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AH3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AI3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AJ3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AK3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AL3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AM3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AN3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AO3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AP3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AQ3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AR3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AS3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AT3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AU3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AV3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AW3" s="5" t="str">
+      <c r="AV3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AW3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AX3" s="5" t="str">
+      <c r="AX3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="AY3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="AZ3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BA3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BB3" s="5" t="str">
+      <c r="AY3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="AZ3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BA3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BB3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="BC3" s="5" t="str">
+      <c r="BC3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="BD3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BE3" s="5" t="str">
+      <c r="BD3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BE3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="BF3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BG3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BH3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BI3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="BJ3" s="5" t="str">
+      <c r="BF3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BG3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BH3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BI3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="BJ3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="B4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="C4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="D4" s="5" t="str">
+      <c r="A4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="B4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="C4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="D4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="F4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="G4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="H4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="I4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="J4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="K4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="L4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="M4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="N4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="O4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="P4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="Q4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="R4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="S4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="T4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="U4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="V4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="W4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="X4" s="5" t="str">
+      <c r="E4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="F4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="G4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="H4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="I4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="J4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="K4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="L4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="M4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="N4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="O4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="P4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="Q4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="R4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="S4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="T4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="U4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="V4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="W4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="X4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="Y4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="Z4" s="5" t="str">
+      <c r="Y4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="Z4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="AA4" s="5" t="str">
+      <c r="AA4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="AB4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AC4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AD4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AE4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AF4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AG4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AH4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AI4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AJ4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AK4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AL4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AM4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AN4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AO4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AP4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AQ4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AR4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AS4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AT4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AU4" s="5" t="str">
+      <c r="AB4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AC4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AD4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AE4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AF4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AG4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AH4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AI4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AJ4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AK4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AL4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AM4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AN4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AO4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AP4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AQ4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AR4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AS4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AT4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AU4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="AV4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AW4" s="5" t="str">
+      <c r="AV4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AW4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="AX4" s="5" t="str">
+      <c r="AX4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="AY4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="AZ4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BA4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BB4" s="5" t="str">
+      <c r="AY4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="AZ4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BA4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BB4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="BC4" s="5" t="str">
+      <c r="BC4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="BD4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BE4" s="5" t="str">
+      <c r="BD4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BE4" s="6" t="str">
         <v>8</v>
       </c>
-      <c r="BF4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BG4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BH4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BI4" s="5" t="str">
-        <v>50</v>
-      </c>
-      <c r="BJ4" s="5" t="str">
+      <c r="BF4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BG4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BH4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BI4" s="6" t="str">
+        <v>50</v>
+      </c>
+      <c r="BJ4" s="6" t="str">
         <v>50</v>
       </c>
     </row>

</xml_diff>